<commit_message>
fix tone parsing + lh reversal
</commit_message>
<xml_diff>
--- a/szeyap-api/src/szeyapapi/data/initials_finals.xlsx
+++ b/szeyap-api/src/szeyapapi/data/initials_finals.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="2044">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="2045">
   <si>
     <t>(none)</t>
   </si>
@@ -4963,6 +4963,9 @@
     <t>x(e)i</t>
   </si>
   <si>
+    <t>chi</t>
+  </si>
+  <si>
     <t>eo</t>
   </si>
   <si>
@@ -5311,9 +5314,6 @@
     <t>ngi</t>
   </si>
   <si>
-    <t>chi</t>
-  </si>
-  <si>
     <t>xiu</t>
   </si>
   <si>
@@ -5878,6 +5878,9 @@
     <t>Notes: There are many little dialectal differences that can be added later as this dictionary will be used mainly by people who don't use the standard accent or a romanization system. For example, 用 may be written as zung for some varieties, 菠蘿包 may be vuo luo vao, and 婆婆 as hu hu. There are orthographic accents as well, such as sh-/ch- for s-/c-, -ee for -i, w- for -v, gn- for ng-, hl- for lh-, which are not covered by the existing dictionaries, so we need to take that into consideration as well. See other file for initial, tone, final, variants</t>
   </si>
   <si>
+    <t>Status</t>
+  </si>
+  <si>
     <t>INPUT</t>
   </si>
   <si>
@@ -5890,7 +5893,7 @@
     <t>OUTPUT</t>
   </si>
   <si>
-    <t>Convert ei to (e)i before search</t>
+    <t>OK</t>
   </si>
   <si>
     <t>neihau</t>
@@ -6626,7 +6629,7 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -6779,6 +6782,9 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="26" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="3" borderId="14" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
@@ -16761,10 +16767,18 @@
       <c r="P14" t="s" s="5">
         <v>241</v>
       </c>
-      <c r="Q14" s="10"/>
-      <c r="R14" s="10"/>
-      <c r="S14" s="10"/>
-      <c r="T14" s="10"/>
+      <c r="Q14" t="s" s="5">
+        <v>242</v>
+      </c>
+      <c r="R14" t="s" s="5">
+        <v>243</v>
+      </c>
+      <c r="S14" t="s" s="5">
+        <v>244</v>
+      </c>
+      <c r="T14" t="s" s="5">
+        <v>245</v>
+      </c>
       <c r="U14" t="s" s="13">
         <v>1267</v>
       </c>
@@ -20625,10 +20639,18 @@
       <c r="P14" t="s" s="5">
         <v>241</v>
       </c>
-      <c r="Q14" s="10"/>
-      <c r="R14" s="10"/>
-      <c r="S14" s="10"/>
-      <c r="T14" s="10"/>
+      <c r="Q14" t="s" s="5">
+        <v>887</v>
+      </c>
+      <c r="R14" t="s" s="5">
+        <v>1648</v>
+      </c>
+      <c r="S14" t="s" s="5">
+        <v>244</v>
+      </c>
+      <c r="T14" t="s" s="5">
+        <v>245</v>
+      </c>
       <c r="U14" t="s" s="13">
         <v>1267</v>
       </c>
@@ -20654,64 +20676,64 @@
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" t="s" s="3">
-        <v>1648</v>
+        <v>1649</v>
       </c>
       <c r="B15" t="s" s="5">
-        <v>1648</v>
+        <v>1649</v>
       </c>
       <c r="C15" t="s" s="5">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="D15" t="s" s="5">
-        <v>1650</v>
+        <v>1651</v>
       </c>
       <c r="E15" t="s" s="5">
-        <v>1651</v>
+        <v>1652</v>
       </c>
       <c r="F15" t="s" s="5">
-        <v>1652</v>
+        <v>1653</v>
       </c>
       <c r="G15" t="s" s="5">
-        <v>1653</v>
+        <v>1654</v>
       </c>
       <c r="H15" t="s" s="5">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="I15" t="s" s="5">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="J15" t="s" s="5">
-        <v>1656</v>
+        <v>1657</v>
       </c>
       <c r="K15" t="s" s="5">
-        <v>1657</v>
+        <v>1658</v>
       </c>
       <c r="L15" t="s" s="5">
-        <v>1658</v>
+        <v>1659</v>
       </c>
       <c r="M15" t="s" s="5">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="N15" t="s" s="5">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="O15" t="s" s="5">
-        <v>1661</v>
+        <v>1662</v>
       </c>
       <c r="P15" t="s" s="5">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="Q15" t="s" s="5">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="R15" t="s" s="5">
-        <v>1664</v>
+        <v>1665</v>
       </c>
       <c r="S15" t="s" s="5">
-        <v>1665</v>
+        <v>1666</v>
       </c>
       <c r="T15" t="s" s="5">
-        <v>1666</v>
+        <v>1667</v>
       </c>
       <c r="U15" s="7"/>
       <c r="V15" s="9"/>
@@ -20736,64 +20758,64 @@
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" t="s" s="3">
-        <v>1667</v>
+        <v>1668</v>
       </c>
       <c r="B16" t="s" s="5">
-        <v>1667</v>
+        <v>1668</v>
       </c>
       <c r="C16" t="s" s="5">
-        <v>1668</v>
+        <v>1669</v>
       </c>
       <c r="D16" t="s" s="5">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="E16" t="s" s="5">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="F16" t="s" s="5">
-        <v>1671</v>
+        <v>1672</v>
       </c>
       <c r="G16" t="s" s="5">
-        <v>1672</v>
+        <v>1673</v>
       </c>
       <c r="H16" t="s" s="5">
-        <v>1673</v>
+        <v>1674</v>
       </c>
       <c r="I16" t="s" s="5">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J16" t="s" s="5">
-        <v>1675</v>
+        <v>1676</v>
       </c>
       <c r="K16" t="s" s="5">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="L16" t="s" s="5">
-        <v>1677</v>
+        <v>1678</v>
       </c>
       <c r="M16" t="s" s="5">
-        <v>1678</v>
+        <v>1679</v>
       </c>
       <c r="N16" t="s" s="5">
-        <v>1679</v>
+        <v>1680</v>
       </c>
       <c r="O16" t="s" s="5">
-        <v>1680</v>
+        <v>1681</v>
       </c>
       <c r="P16" t="s" s="5">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="Q16" t="s" s="5">
-        <v>1682</v>
+        <v>1683</v>
       </c>
       <c r="R16" t="s" s="5">
-        <v>1683</v>
+        <v>1684</v>
       </c>
       <c r="S16" t="s" s="5">
-        <v>1684</v>
+        <v>1685</v>
       </c>
       <c r="T16" t="s" s="5">
-        <v>1685</v>
+        <v>1686</v>
       </c>
       <c r="U16" s="7"/>
       <c r="V16" s="9"/>
@@ -20818,64 +20840,64 @@
     </row>
     <row r="17" ht="14.25" customHeight="1">
       <c r="A17" t="s" s="11">
-        <v>1686</v>
+        <v>1687</v>
       </c>
       <c r="B17" t="s" s="5">
-        <v>1686</v>
+        <v>1687</v>
       </c>
       <c r="C17" t="s" s="5">
-        <v>1687</v>
+        <v>1688</v>
       </c>
       <c r="D17" t="s" s="5">
-        <v>1688</v>
+        <v>1689</v>
       </c>
       <c r="E17" t="s" s="5">
-        <v>1689</v>
+        <v>1690</v>
       </c>
       <c r="F17" t="s" s="5">
-        <v>1690</v>
+        <v>1691</v>
       </c>
       <c r="G17" t="s" s="5">
-        <v>1691</v>
+        <v>1692</v>
       </c>
       <c r="H17" t="s" s="5">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="I17" t="s" s="5">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="J17" t="s" s="5">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="K17" t="s" s="5">
-        <v>1695</v>
+        <v>1696</v>
       </c>
       <c r="L17" t="s" s="5">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="M17" t="s" s="5">
-        <v>1697</v>
+        <v>1698</v>
       </c>
       <c r="N17" t="s" s="5">
-        <v>1698</v>
+        <v>1699</v>
       </c>
       <c r="O17" t="s" s="5">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="P17" t="s" s="5">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="Q17" t="s" s="5">
-        <v>1701</v>
+        <v>1702</v>
       </c>
       <c r="R17" t="s" s="5">
-        <v>1702</v>
+        <v>1703</v>
       </c>
       <c r="S17" t="s" s="5">
-        <v>1703</v>
+        <v>1704</v>
       </c>
       <c r="T17" t="s" s="5">
-        <v>1704</v>
+        <v>1705</v>
       </c>
       <c r="U17" s="7"/>
       <c r="V17" s="9"/>
@@ -20933,7 +20955,7 @@
         <v>293</v>
       </c>
       <c r="L18" t="s" s="5">
-        <v>1705</v>
+        <v>1706</v>
       </c>
       <c r="M18" t="s" s="5">
         <v>295</v>
@@ -20951,7 +20973,7 @@
         <v>894</v>
       </c>
       <c r="R18" t="s" s="5">
-        <v>1706</v>
+        <v>1707</v>
       </c>
       <c r="S18" t="s" s="5">
         <v>301</v>
@@ -20982,64 +21004,64 @@
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" t="s" s="3">
-        <v>1707</v>
+        <v>1708</v>
       </c>
       <c r="B19" t="s" s="5">
-        <v>1707</v>
+        <v>1708</v>
       </c>
       <c r="C19" t="s" s="5">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="D19" t="s" s="5">
-        <v>1709</v>
+        <v>1710</v>
       </c>
       <c r="E19" t="s" s="5">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="F19" t="s" s="5">
-        <v>1711</v>
+        <v>1712</v>
       </c>
       <c r="G19" t="s" s="5">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="H19" t="s" s="5">
-        <v>1713</v>
+        <v>1714</v>
       </c>
       <c r="I19" t="s" s="5">
-        <v>1714</v>
+        <v>1715</v>
       </c>
       <c r="J19" t="s" s="5">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="K19" t="s" s="5">
-        <v>1716</v>
+        <v>1717</v>
       </c>
       <c r="L19" t="s" s="5">
-        <v>1717</v>
+        <v>1718</v>
       </c>
       <c r="M19" t="s" s="5">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="N19" t="s" s="5">
-        <v>1719</v>
+        <v>1720</v>
       </c>
       <c r="O19" t="s" s="5">
-        <v>1720</v>
+        <v>1721</v>
       </c>
       <c r="P19" t="s" s="5">
-        <v>1721</v>
+        <v>1722</v>
       </c>
       <c r="Q19" t="s" s="5">
-        <v>1722</v>
+        <v>1723</v>
       </c>
       <c r="R19" t="s" s="5">
-        <v>1723</v>
+        <v>1724</v>
       </c>
       <c r="S19" t="s" s="5">
-        <v>1724</v>
+        <v>1725</v>
       </c>
       <c r="T19" t="s" s="5">
-        <v>1725</v>
+        <v>1726</v>
       </c>
       <c r="U19" s="7"/>
       <c r="V19" s="9"/>
@@ -21064,64 +21086,64 @@
     </row>
     <row r="20" ht="14.25" customHeight="1">
       <c r="A20" t="s" s="11">
-        <v>1726</v>
+        <v>1727</v>
       </c>
       <c r="B20" t="s" s="5">
-        <v>1726</v>
+        <v>1727</v>
       </c>
       <c r="C20" t="s" s="5">
-        <v>1727</v>
+        <v>1728</v>
       </c>
       <c r="D20" t="s" s="5">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="E20" t="s" s="5">
-        <v>1729</v>
+        <v>1730</v>
       </c>
       <c r="F20" t="s" s="5">
-        <v>1730</v>
+        <v>1731</v>
       </c>
       <c r="G20" t="s" s="5">
-        <v>1731</v>
+        <v>1732</v>
       </c>
       <c r="H20" t="s" s="5">
-        <v>1732</v>
+        <v>1733</v>
       </c>
       <c r="I20" t="s" s="5">
-        <v>1733</v>
+        <v>1734</v>
       </c>
       <c r="J20" t="s" s="5">
-        <v>1734</v>
+        <v>1735</v>
       </c>
       <c r="K20" t="s" s="5">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="L20" t="s" s="5">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="M20" t="s" s="5">
-        <v>1737</v>
+        <v>1738</v>
       </c>
       <c r="N20" t="s" s="5">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="O20" t="s" s="5">
-        <v>1739</v>
+        <v>1740</v>
       </c>
       <c r="P20" t="s" s="5">
-        <v>1740</v>
+        <v>1741</v>
       </c>
       <c r="Q20" t="s" s="5">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="R20" t="s" s="5">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="S20" t="s" s="5">
-        <v>1743</v>
+        <v>1744</v>
       </c>
       <c r="T20" t="s" s="5">
-        <v>1744</v>
+        <v>1745</v>
       </c>
       <c r="U20" s="7"/>
       <c r="V20" s="9"/>
@@ -21179,7 +21201,7 @@
         <v>331</v>
       </c>
       <c r="L21" t="s" s="5">
-        <v>1745</v>
+        <v>1746</v>
       </c>
       <c r="M21" t="s" s="5">
         <v>333</v>
@@ -21194,10 +21216,10 @@
         <v>336</v>
       </c>
       <c r="Q21" t="s" s="5">
-        <v>1746</v>
+        <v>1747</v>
       </c>
       <c r="R21" t="s" s="5">
-        <v>1747</v>
+        <v>1748</v>
       </c>
       <c r="S21" t="s" s="5">
         <v>339</v>
@@ -21307,7 +21329,7 @@
         <v>350</v>
       </c>
       <c r="L23" t="s" s="5">
-        <v>1748</v>
+        <v>1749</v>
       </c>
       <c r="M23" t="s" s="5">
         <v>352</v>
@@ -21325,7 +21347,7 @@
         <v>935</v>
       </c>
       <c r="R23" t="s" s="5">
-        <v>1749</v>
+        <v>1750</v>
       </c>
       <c r="S23" t="s" s="5">
         <v>358</v>
@@ -21389,7 +21411,7 @@
         <v>369</v>
       </c>
       <c r="L24" t="s" s="5">
-        <v>1750</v>
+        <v>1751</v>
       </c>
       <c r="M24" t="s" s="5">
         <v>371</v>
@@ -21407,7 +21429,7 @@
         <v>937</v>
       </c>
       <c r="R24" t="s" s="5">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="S24" t="s" s="5">
         <v>377</v>
@@ -21471,7 +21493,7 @@
         <v>388</v>
       </c>
       <c r="L25" t="s" s="5">
-        <v>1752</v>
+        <v>1753</v>
       </c>
       <c r="M25" t="s" s="5">
         <v>390</v>
@@ -21489,7 +21511,7 @@
         <v>939</v>
       </c>
       <c r="R25" t="s" s="5">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="S25" t="s" s="5">
         <v>396</v>
@@ -21553,7 +21575,7 @@
         <v>407</v>
       </c>
       <c r="L26" t="s" s="5">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="M26" t="s" s="5">
         <v>409</v>
@@ -21571,7 +21593,7 @@
         <v>941</v>
       </c>
       <c r="R26" t="s" s="5">
-        <v>1755</v>
+        <v>1756</v>
       </c>
       <c r="S26" t="s" s="5">
         <v>415</v>
@@ -21635,7 +21657,7 @@
         <v>426</v>
       </c>
       <c r="L27" t="s" s="5">
-        <v>1756</v>
+        <v>1757</v>
       </c>
       <c r="M27" t="s" s="5">
         <v>428</v>
@@ -21650,10 +21672,10 @@
         <v>431</v>
       </c>
       <c r="Q27" t="s" s="5">
-        <v>1757</v>
+        <v>1758</v>
       </c>
       <c r="R27" t="s" s="5">
-        <v>1758</v>
+        <v>1759</v>
       </c>
       <c r="S27" t="s" s="5">
         <v>434</v>
@@ -21717,7 +21739,7 @@
         <v>445</v>
       </c>
       <c r="L28" t="s" s="5">
-        <v>1759</v>
+        <v>1760</v>
       </c>
       <c r="M28" t="s" s="5">
         <v>447</v>
@@ -21732,10 +21754,10 @@
         <v>450</v>
       </c>
       <c r="Q28" t="s" s="5">
-        <v>1760</v>
+        <v>1761</v>
       </c>
       <c r="R28" t="s" s="5">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="S28" t="s" s="5">
         <v>453</v>
@@ -21799,7 +21821,7 @@
         <v>1522</v>
       </c>
       <c r="L29" t="s" s="5">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="M29" t="s" s="5">
         <v>1524</v>
@@ -21808,7 +21830,7 @@
         <v>1525</v>
       </c>
       <c r="O29" t="s" s="5">
-        <v>1763</v>
+        <v>1764</v>
       </c>
       <c r="P29" t="s" s="5">
         <v>1527</v>
@@ -21817,7 +21839,7 @@
         <v>887</v>
       </c>
       <c r="R29" t="s" s="5">
-        <v>1764</v>
+        <v>1648</v>
       </c>
       <c r="S29" t="s" s="5">
         <v>244</v>
@@ -22947,7 +22969,7 @@
         <v>350</v>
       </c>
       <c r="L43" t="s" s="5">
-        <v>1748</v>
+        <v>1749</v>
       </c>
       <c r="M43" t="s" s="5">
         <v>352</v>
@@ -22965,7 +22987,7 @@
         <v>935</v>
       </c>
       <c r="R43" t="s" s="5">
-        <v>1749</v>
+        <v>1750</v>
       </c>
       <c r="S43" t="s" s="5">
         <v>358</v>
@@ -24496,7 +24518,7 @@
         <v>1897</v>
       </c>
       <c r="S14" t="s" s="5">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="T14" t="s" s="5">
         <v>245</v>
@@ -25692,7 +25714,7 @@
         <v>1897</v>
       </c>
       <c r="S29" t="s" s="5">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="T29" t="s" s="5">
         <v>245</v>
@@ -27625,242 +27647,250 @@
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
-      <c r="A3" s="46"/>
-      <c r="B3" t="s" s="51">
+      <c r="A3" t="s" s="51">
         <v>1953</v>
       </c>
-      <c r="C3" t="s" s="51">
+      <c r="B3" t="s" s="52">
         <v>1954</v>
       </c>
-      <c r="D3" t="s" s="51">
+      <c r="C3" t="s" s="52">
         <v>1955</v>
       </c>
-      <c r="E3" t="s" s="52">
+      <c r="D3" t="s" s="52">
         <v>1956</v>
       </c>
-      <c r="F3" s="53"/>
+      <c r="E3" t="s" s="53">
+        <v>1957</v>
+      </c>
+      <c r="F3" s="54"/>
     </row>
     <row r="4" ht="14.25" customHeight="1">
-      <c r="A4" t="s" s="54">
-        <v>1957</v>
-      </c>
-      <c r="B4" t="s" s="55">
+      <c r="A4" t="s" s="55">
         <v>1958</v>
       </c>
-      <c r="C4" t="s" s="55">
+      <c r="B4" t="s" s="56">
         <v>1959</v>
       </c>
-      <c r="D4" t="s" s="55">
+      <c r="C4" t="s" s="56">
         <v>1960</v>
       </c>
-      <c r="E4" s="56"/>
+      <c r="D4" t="s" s="56">
+        <v>1961</v>
+      </c>
+      <c r="E4" s="57"/>
       <c r="F4" s="9"/>
     </row>
     <row r="5" ht="14.25" customHeight="1">
-      <c r="A5" s="9"/>
-      <c r="B5" t="s" s="54">
-        <v>1961</v>
-      </c>
-      <c r="C5" t="s" s="54">
+      <c r="A5" t="s" s="55">
+        <v>1958</v>
+      </c>
+      <c r="B5" t="s" s="55">
         <v>1962</v>
       </c>
-      <c r="D5" t="s" s="54">
+      <c r="C5" t="s" s="55">
         <v>1963</v>
+      </c>
+      <c r="D5" t="s" s="55">
+        <v>1964</v>
       </c>
       <c r="E5" s="9"/>
       <c r="F5" s="9"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
-      <c r="A6" s="9"/>
-      <c r="B6" t="s" s="54">
+      <c r="A6" t="s" s="55">
+        <v>1958</v>
+      </c>
+      <c r="B6" t="s" s="55">
+        <v>1965</v>
+      </c>
+      <c r="C6" t="s" s="55">
+        <v>1966</v>
+      </c>
+      <c r="D6" t="s" s="55">
         <v>1964</v>
-      </c>
-      <c r="C6" t="s" s="54">
-        <v>1965</v>
-      </c>
-      <c r="D6" t="s" s="54">
-        <v>1963</v>
       </c>
       <c r="E6" s="9"/>
       <c r="F6" s="9"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
-      <c r="A7" s="9"/>
-      <c r="B7" t="s" s="54">
-        <v>1966</v>
-      </c>
-      <c r="C7" t="s" s="54">
+      <c r="A7" t="s" s="55">
+        <v>1958</v>
+      </c>
+      <c r="B7" t="s" s="55">
         <v>1967</v>
       </c>
-      <c r="D7" t="s" s="54">
+      <c r="C7" t="s" s="55">
         <v>1968</v>
+      </c>
+      <c r="D7" t="s" s="55">
+        <v>1969</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
     </row>
     <row r="8" ht="14.25" customHeight="1">
       <c r="A8" s="9"/>
-      <c r="B8" t="s" s="54">
-        <v>1969</v>
-      </c>
-      <c r="C8" t="s" s="54">
+      <c r="B8" t="s" s="55">
         <v>1970</v>
       </c>
-      <c r="D8" t="s" s="54">
+      <c r="C8" t="s" s="55">
         <v>1971</v>
+      </c>
+      <c r="D8" t="s" s="55">
+        <v>1972</v>
       </c>
       <c r="E8" s="9"/>
       <c r="F8" s="9"/>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="9"/>
-      <c r="B9" t="s" s="54">
-        <v>1972</v>
-      </c>
-      <c r="C9" t="s" s="54">
+      <c r="B9" t="s" s="55">
         <v>1973</v>
       </c>
-      <c r="D9" t="s" s="54">
+      <c r="C9" t="s" s="55">
         <v>1974</v>
+      </c>
+      <c r="D9" t="s" s="55">
+        <v>1975</v>
       </c>
       <c r="E9" s="9"/>
       <c r="F9" s="9"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="9"/>
-      <c r="B10" t="s" s="54">
-        <v>1975</v>
-      </c>
-      <c r="C10" t="s" s="54">
+      <c r="B10" t="s" s="55">
         <v>1976</v>
       </c>
-      <c r="D10" t="s" s="54">
+      <c r="C10" t="s" s="55">
         <v>1977</v>
+      </c>
+      <c r="D10" t="s" s="55">
+        <v>1978</v>
       </c>
       <c r="E10" s="9"/>
       <c r="F10" s="9"/>
     </row>
     <row r="11" ht="14.25" customHeight="1">
       <c r="A11" s="9"/>
-      <c r="B11" t="s" s="54">
-        <v>1978</v>
-      </c>
-      <c r="C11" t="s" s="54">
-        <v>1967</v>
-      </c>
-      <c r="D11" t="s" s="54">
+      <c r="B11" t="s" s="55">
         <v>1979</v>
+      </c>
+      <c r="C11" t="s" s="55">
+        <v>1968</v>
+      </c>
+      <c r="D11" t="s" s="55">
+        <v>1980</v>
       </c>
       <c r="E11" s="9"/>
       <c r="F11" s="9"/>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="9"/>
-      <c r="B12" t="s" s="54">
-        <v>1980</v>
-      </c>
-      <c r="C12" t="s" s="54">
+      <c r="B12" t="s" s="55">
         <v>1981</v>
       </c>
-      <c r="D12" t="s" s="54">
+      <c r="C12" t="s" s="55">
         <v>1982</v>
+      </c>
+      <c r="D12" t="s" s="55">
+        <v>1983</v>
       </c>
       <c r="E12" s="9"/>
       <c r="F12" s="9"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="9"/>
-      <c r="B13" t="s" s="54">
-        <v>1983</v>
-      </c>
-      <c r="C13" t="s" s="54">
-        <v>1967</v>
-      </c>
-      <c r="D13" t="s" s="54">
+      <c r="B13" t="s" s="55">
         <v>1984</v>
+      </c>
+      <c r="C13" t="s" s="55">
+        <v>1968</v>
+      </c>
+      <c r="D13" t="s" s="55">
+        <v>1985</v>
       </c>
       <c r="E13" s="9"/>
       <c r="F13" s="9"/>
     </row>
     <row r="14" ht="14.25" customHeight="1">
       <c r="A14" s="9"/>
-      <c r="B14" t="s" s="54">
-        <v>1985</v>
-      </c>
-      <c r="C14" t="s" s="54">
+      <c r="B14" t="s" s="55">
         <v>1986</v>
       </c>
-      <c r="D14" t="s" s="54">
+      <c r="C14" t="s" s="55">
         <v>1987</v>
+      </c>
+      <c r="D14" t="s" s="55">
+        <v>1988</v>
       </c>
       <c r="E14" s="9"/>
       <c r="F14" s="9"/>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="9"/>
-      <c r="B15" t="s" s="54">
+      <c r="B15" t="s" s="55">
         <v>233</v>
       </c>
-      <c r="C15" t="s" s="54">
-        <v>1988</v>
-      </c>
-      <c r="D15" t="s" s="54">
+      <c r="C15" t="s" s="55">
         <v>1989</v>
+      </c>
+      <c r="D15" t="s" s="55">
+        <v>1990</v>
       </c>
       <c r="E15" s="9"/>
       <c r="F15" s="9"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="9"/>
-      <c r="B16" t="s" s="54">
-        <v>1990</v>
-      </c>
-      <c r="C16" t="s" s="54">
+      <c r="B16" t="s" s="55">
         <v>1991</v>
       </c>
-      <c r="D16" t="s" s="54">
+      <c r="C16" t="s" s="55">
         <v>1992</v>
       </c>
-      <c r="E16" t="s" s="54">
+      <c r="D16" t="s" s="55">
         <v>1993</v>
+      </c>
+      <c r="E16" t="s" s="55">
+        <v>1994</v>
       </c>
       <c r="F16" s="9"/>
     </row>
     <row r="17" ht="14.25" customHeight="1">
       <c r="A17" s="9"/>
-      <c r="B17" t="s" s="54">
+      <c r="B17" t="s" s="55">
+        <v>1995</v>
+      </c>
+      <c r="C17" t="s" s="55">
+        <v>1996</v>
+      </c>
+      <c r="D17" s="9"/>
+      <c r="E17" t="s" s="55">
         <v>1994</v>
-      </c>
-      <c r="C17" t="s" s="54">
-        <v>1995</v>
-      </c>
-      <c r="D17" s="9"/>
-      <c r="E17" t="s" s="54">
-        <v>1993</v>
       </c>
       <c r="F17" s="9"/>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="9"/>
-      <c r="B18" t="s" s="54">
+      <c r="B18" t="s" s="55">
+        <v>1997</v>
+      </c>
+      <c r="C18" t="s" s="55">
         <v>1996</v>
       </c>
-      <c r="C18" t="s" s="54">
-        <v>1995</v>
-      </c>
       <c r="D18" s="9"/>
-      <c r="E18" t="s" s="54">
-        <v>1993</v>
+      <c r="E18" t="s" s="55">
+        <v>1994</v>
       </c>
       <c r="F18" s="9"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="9"/>
-      <c r="B19" t="s" s="54">
-        <v>1997</v>
-      </c>
-      <c r="C19" t="s" s="54">
+      <c r="B19" t="s" s="55">
         <v>1998</v>
+      </c>
+      <c r="C19" t="s" s="55">
+        <v>1999</v>
       </c>
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
@@ -27868,39 +27898,39 @@
     </row>
     <row r="20" ht="14.25" customHeight="1">
       <c r="A20" s="9"/>
-      <c r="B20" t="s" s="54">
+      <c r="B20" t="s" s="55">
         <v>354</v>
       </c>
-      <c r="C20" t="s" s="54">
-        <v>1999</v>
-      </c>
-      <c r="D20" t="s" s="54">
+      <c r="C20" t="s" s="55">
         <v>2000</v>
+      </c>
+      <c r="D20" t="s" s="55">
+        <v>2001</v>
       </c>
       <c r="E20" s="9"/>
       <c r="F20" s="9"/>
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="9"/>
-      <c r="B21" t="s" s="54">
-        <v>2001</v>
-      </c>
-      <c r="C21" t="s" s="54">
+      <c r="B21" t="s" s="55">
         <v>2002</v>
       </c>
-      <c r="D21" t="s" s="54">
+      <c r="C21" t="s" s="55">
         <v>2003</v>
+      </c>
+      <c r="D21" t="s" s="55">
+        <v>2004</v>
       </c>
       <c r="E21" s="9"/>
       <c r="F21" s="9"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="9"/>
-      <c r="B22" t="s" s="54">
-        <v>2004</v>
-      </c>
-      <c r="C22" t="s" s="54">
+      <c r="B22" t="s" s="55">
         <v>2005</v>
+      </c>
+      <c r="C22" t="s" s="55">
+        <v>2006</v>
       </c>
       <c r="D22" s="9"/>
       <c r="E22" s="9"/>
@@ -27908,122 +27938,122 @@
     </row>
     <row r="23" ht="14.25" customHeight="1">
       <c r="A23" s="9"/>
-      <c r="B23" t="s" s="54">
-        <v>2006</v>
-      </c>
-      <c r="C23" t="s" s="54">
+      <c r="B23" t="s" s="55">
         <v>2007</v>
       </c>
-      <c r="D23" t="s" s="54">
+      <c r="C23" t="s" s="55">
         <v>2008</v>
+      </c>
+      <c r="D23" t="s" s="55">
+        <v>2009</v>
       </c>
       <c r="E23" s="9"/>
       <c r="F23" s="9"/>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="9"/>
-      <c r="B24" t="s" s="54">
-        <v>2009</v>
+      <c r="B24" t="s" s="55">
+        <v>2010</v>
       </c>
       <c r="C24" s="9"/>
-      <c r="D24" t="s" s="54">
-        <v>2010</v>
+      <c r="D24" t="s" s="55">
+        <v>2011</v>
       </c>
       <c r="E24" s="9"/>
       <c r="F24" s="9"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="9"/>
-      <c r="B25" t="s" s="54">
-        <v>2011</v>
+      <c r="B25" t="s" s="55">
+        <v>2012</v>
       </c>
       <c r="C25" s="9"/>
-      <c r="D25" t="s" s="54">
-        <v>2012</v>
+      <c r="D25" t="s" s="55">
+        <v>2013</v>
       </c>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
     </row>
     <row r="26" ht="14.25" customHeight="1">
       <c r="A26" s="9"/>
-      <c r="B26" t="s" s="54">
+      <c r="B26" t="s" s="55">
         <v>285</v>
       </c>
-      <c r="C26" t="s" s="54">
-        <v>2013</v>
-      </c>
-      <c r="D26" t="s" s="54">
+      <c r="C26" t="s" s="55">
         <v>2014</v>
+      </c>
+      <c r="D26" t="s" s="55">
+        <v>2015</v>
       </c>
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="9"/>
-      <c r="B27" t="s" s="54">
+      <c r="B27" t="s" s="55">
         <v>339</v>
       </c>
-      <c r="C27" t="s" s="54">
-        <v>2013</v>
-      </c>
-      <c r="D27" t="s" s="54">
-        <v>2015</v>
+      <c r="C27" t="s" s="55">
+        <v>2014</v>
+      </c>
+      <c r="D27" t="s" s="55">
+        <v>2016</v>
       </c>
       <c r="E27" s="9"/>
       <c r="F27" s="9"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="9"/>
-      <c r="B28" t="s" s="54">
+      <c r="B28" t="s" s="55">
         <v>705</v>
       </c>
-      <c r="C28" t="s" s="54">
-        <v>2016</v>
-      </c>
-      <c r="D28" t="s" s="54">
+      <c r="C28" t="s" s="55">
         <v>2017</v>
+      </c>
+      <c r="D28" t="s" s="55">
+        <v>2018</v>
       </c>
       <c r="E28" s="9"/>
       <c r="F28" s="9"/>
     </row>
     <row r="29" ht="14.25" customHeight="1">
       <c r="A29" s="9"/>
-      <c r="B29" t="s" s="54">
-        <v>2018</v>
-      </c>
-      <c r="C29" t="s" s="54">
-        <v>2016</v>
-      </c>
-      <c r="D29" t="s" s="54">
+      <c r="B29" t="s" s="55">
         <v>2019</v>
+      </c>
+      <c r="C29" t="s" s="55">
+        <v>2017</v>
+      </c>
+      <c r="D29" t="s" s="55">
+        <v>2020</v>
       </c>
       <c r="E29" s="9"/>
       <c r="F29" s="9"/>
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="9"/>
-      <c r="B30" t="s" s="54">
-        <v>2020</v>
-      </c>
-      <c r="C30" t="s" s="54">
-        <v>2016</v>
-      </c>
-      <c r="D30" t="s" s="54">
+      <c r="B30" t="s" s="55">
         <v>2021</v>
+      </c>
+      <c r="C30" t="s" s="55">
+        <v>2017</v>
+      </c>
+      <c r="D30" t="s" s="55">
+        <v>2022</v>
       </c>
       <c r="E30" s="9"/>
       <c r="F30" s="9"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="9"/>
-      <c r="B31" t="s" s="54">
-        <v>2022</v>
-      </c>
-      <c r="C31" t="s" s="54">
-        <v>2016</v>
-      </c>
-      <c r="D31" t="s" s="54">
+      <c r="B31" t="s" s="55">
         <v>2023</v>
+      </c>
+      <c r="C31" t="s" s="55">
+        <v>2017</v>
+      </c>
+      <c r="D31" t="s" s="55">
+        <v>2024</v>
       </c>
       <c r="E31" s="9"/>
       <c r="F31" s="9"/>
@@ -28038,8 +28068,8 @@
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="46"/>
-      <c r="B33" t="s" s="57">
-        <v>2024</v>
+      <c r="B33" t="s" s="58">
+        <v>2025</v>
       </c>
       <c r="C33" s="48"/>
       <c r="D33" s="49"/>
@@ -28048,110 +28078,110 @@
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="46"/>
-      <c r="B34" t="s" s="52">
-        <v>1953</v>
-      </c>
-      <c r="C34" t="s" s="52">
+      <c r="B34" t="s" s="53">
         <v>1954</v>
       </c>
-      <c r="D34" t="s" s="52">
+      <c r="C34" t="s" s="53">
         <v>1955</v>
       </c>
-      <c r="E34" t="s" s="52">
+      <c r="D34" t="s" s="53">
         <v>1956</v>
       </c>
-      <c r="F34" s="53"/>
+      <c r="E34" t="s" s="53">
+        <v>1957</v>
+      </c>
+      <c r="F34" s="54"/>
     </row>
     <row r="35" ht="14.25" customHeight="1">
       <c r="A35" s="9"/>
-      <c r="B35" t="s" s="55">
-        <v>2025</v>
-      </c>
-      <c r="C35" t="s" s="55">
+      <c r="B35" t="s" s="56">
         <v>2026</v>
       </c>
-      <c r="D35" t="s" s="55">
+      <c r="C35" t="s" s="56">
         <v>2027</v>
       </c>
-      <c r="E35" t="s" s="55">
+      <c r="D35" t="s" s="56">
         <v>2028</v>
+      </c>
+      <c r="E35" t="s" s="56">
+        <v>2029</v>
       </c>
       <c r="F35" s="9"/>
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="9"/>
-      <c r="B36" t="s" s="54">
-        <v>1762</v>
-      </c>
-      <c r="C36" t="s" s="54">
+      <c r="B36" t="s" s="55">
+        <v>1763</v>
+      </c>
+      <c r="C36" t="s" s="55">
+        <v>2030</v>
+      </c>
+      <c r="D36" t="s" s="55">
+        <v>2031</v>
+      </c>
+      <c r="E36" t="s" s="55">
         <v>2029</v>
-      </c>
-      <c r="D36" t="s" s="54">
-        <v>2030</v>
-      </c>
-      <c r="E36" t="s" s="54">
-        <v>2028</v>
       </c>
       <c r="F36" s="9"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="9"/>
-      <c r="B37" t="s" s="54">
-        <v>2031</v>
-      </c>
-      <c r="C37" t="s" s="54">
+      <c r="B37" t="s" s="55">
         <v>2032</v>
       </c>
-      <c r="D37" t="s" s="54">
+      <c r="C37" t="s" s="55">
         <v>2033</v>
       </c>
-      <c r="E37" t="s" s="54">
-        <v>1993</v>
+      <c r="D37" t="s" s="55">
+        <v>2034</v>
+      </c>
+      <c r="E37" t="s" s="55">
+        <v>1994</v>
       </c>
       <c r="F37" s="9"/>
     </row>
     <row r="38" ht="14.25" customHeight="1">
       <c r="A38" s="9"/>
-      <c r="B38" t="s" s="54">
-        <v>2034</v>
-      </c>
-      <c r="C38" t="s" s="54">
+      <c r="B38" t="s" s="55">
         <v>2035</v>
       </c>
-      <c r="D38" t="s" s="54">
-        <v>2035</v>
-      </c>
-      <c r="E38" t="s" s="54">
+      <c r="C38" t="s" s="55">
         <v>2036</v>
+      </c>
+      <c r="D38" t="s" s="55">
+        <v>2036</v>
+      </c>
+      <c r="E38" t="s" s="55">
+        <v>2037</v>
       </c>
       <c r="F38" s="9"/>
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="9"/>
-      <c r="B39" t="s" s="54">
-        <v>2037</v>
-      </c>
-      <c r="C39" t="s" s="54">
+      <c r="B39" t="s" s="55">
         <v>2038</v>
       </c>
-      <c r="D39" t="s" s="54">
+      <c r="C39" t="s" s="55">
         <v>2039</v>
       </c>
-      <c r="E39" t="s" s="58">
+      <c r="D39" t="s" s="55">
         <v>2040</v>
+      </c>
+      <c r="E39" t="s" s="59">
+        <v>2041</v>
       </c>
       <c r="F39" s="9"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="9"/>
-      <c r="B40" t="s" s="54">
-        <v>2041</v>
-      </c>
-      <c r="C40" t="s" s="54">
+      <c r="B40" t="s" s="55">
         <v>2042</v>
       </c>
-      <c r="D40" t="s" s="54">
+      <c r="C40" t="s" s="55">
         <v>2043</v>
+      </c>
+      <c r="D40" t="s" s="55">
+        <v>2044</v>
       </c>
       <c r="E40" s="9"/>
       <c r="F40" s="9"/>

</xml_diff>

<commit_message>
hotfix for parsing SL penyim
</commit_message>
<xml_diff>
--- a/szeyap-api/src/szeyapapi/data/initials_finals.xlsx
+++ b/szeyap-api/src/szeyapapi/data/initials_finals.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="HSR" sheetId="1" state="visible" r:id="rId3"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4840" uniqueCount="2043">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4840" uniqueCount="2028">
   <si>
     <t xml:space="preserve">(none)</t>
   </si>
@@ -3946,61 +3946,61 @@
     <t xml:space="preserve">yəm</t>
   </si>
   <si>
-    <t xml:space="preserve">ɛɪn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bɛɪn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pɛɪn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mɛɪn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fɛɪn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">vɛɪn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dɛɪn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tɛɪn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nɛɪn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lɛɪn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ɬɛɪn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gɛɪn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kɛɪn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ŋɛɪn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hɛɪn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dzɛɪn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tsɛɪn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sɛɪn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">yɛɪn</t>
+    <t xml:space="preserve">ein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ɬein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ŋein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dzein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tsein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yein</t>
   </si>
   <si>
     <t xml:space="preserve">ian</t>
@@ -5089,61 +5089,16 @@
     <t xml:space="preserve">yeim</t>
   </si>
   <si>
-    <t xml:space="preserve">ein</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bein</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pein</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mein</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fein</t>
-  </si>
-  <si>
-    <t xml:space="preserve">vein</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dein</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tein</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nein</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lein</t>
-  </si>
-  <si>
     <t xml:space="preserve">xein</t>
   </si>
   <si>
-    <t xml:space="preserve">gein</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kein</t>
-  </si>
-  <si>
     <t xml:space="preserve">ngein</t>
   </si>
   <si>
-    <t xml:space="preserve">hein</t>
-  </si>
-  <si>
     <t xml:space="preserve">jein</t>
   </si>
   <si>
     <t xml:space="preserve">chein</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sein</t>
-  </si>
-  <si>
-    <t xml:space="preserve">yein</t>
   </si>
   <si>
     <t xml:space="preserve">xen</t>
@@ -5685,6 +5640,7 @@
         <sz val="11"/>
         <rFont val="PingFang SC"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">〉</t>
     </r>
@@ -5914,6 +5870,7 @@
         <sz val="11"/>
         <rFont val="PingFang SC"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">用 </t>
     </r>
@@ -5931,6 +5888,7 @@
         <sz val="11"/>
         <rFont val="PingFang SC"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">菠蘿包 </t>
     </r>
@@ -5948,6 +5906,7 @@
         <sz val="11"/>
         <rFont val="PingFang SC"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">婆婆 </t>
     </r>
@@ -6272,6 +6231,7 @@
       <sz val="11"/>
       <name val="PingFang SC"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="20"/>
@@ -6763,10 +6723,10 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AN47"/>
-  <sheetFormatPr defaultColWidth="14.5078125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.515625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="1" style="1" width="8.68"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="41" style="1" width="14.51"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="41" style="1" width="14.52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10638,10 +10598,10 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AN47"/>
-  <sheetFormatPr defaultColWidth="14.5078125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.515625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="1" style="1" width="8.68"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="41" style="1" width="14.51"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="41" style="1" width="14.52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14515,10 +14475,10 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AN47"/>
-  <sheetFormatPr defaultColWidth="14.5078125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.515625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="1" style="1" width="8.68"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="41" style="1" width="14.51"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="41" style="1" width="14.52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18396,10 +18356,10 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AN47"/>
-  <sheetFormatPr defaultColWidth="14.5078125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.515625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="1" style="1" width="8.68"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="41" style="1" width="14.51"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="41" style="1" width="14.52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19752,64 +19712,64 @@
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
+        <v>1306</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>1306</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>1307</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>1308</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>1309</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>1310</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>1311</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>1312</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>1313</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>1314</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>1315</v>
+      </c>
+      <c r="L17" s="3" t="s">
         <v>1687</v>
       </c>
-      <c r="B17" s="3" t="s">
-        <v>1687</v>
-      </c>
-      <c r="C17" s="3" t="s">
+      <c r="M17" s="3" t="s">
+        <v>1317</v>
+      </c>
+      <c r="N17" s="3" t="s">
+        <v>1318</v>
+      </c>
+      <c r="O17" s="3" t="s">
         <v>1688</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="P17" s="3" t="s">
+        <v>1320</v>
+      </c>
+      <c r="Q17" s="3" t="s">
         <v>1689</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="R17" s="3" t="s">
         <v>1690</v>
       </c>
-      <c r="F17" s="3" t="s">
-        <v>1691</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>1692</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>1693</v>
-      </c>
-      <c r="I17" s="3" t="s">
-        <v>1694</v>
-      </c>
-      <c r="J17" s="3" t="s">
-        <v>1695</v>
-      </c>
-      <c r="K17" s="3" t="s">
-        <v>1696</v>
-      </c>
-      <c r="L17" s="3" t="s">
-        <v>1697</v>
-      </c>
-      <c r="M17" s="3" t="s">
-        <v>1698</v>
-      </c>
-      <c r="N17" s="3" t="s">
-        <v>1699</v>
-      </c>
-      <c r="O17" s="3" t="s">
-        <v>1700</v>
-      </c>
-      <c r="P17" s="3" t="s">
-        <v>1701</v>
-      </c>
-      <c r="Q17" s="3" t="s">
-        <v>1702</v>
-      </c>
-      <c r="R17" s="3" t="s">
-        <v>1703</v>
-      </c>
       <c r="S17" s="3" t="s">
-        <v>1704</v>
+        <v>1323</v>
       </c>
       <c r="T17" s="3" t="s">
-        <v>1705</v>
+        <v>1324</v>
       </c>
       <c r="U17" s="4"/>
       <c r="V17" s="4"/>
@@ -19867,7 +19827,7 @@
         <v>293</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>1706</v>
+        <v>1691</v>
       </c>
       <c r="M18" s="3" t="s">
         <v>295</v>
@@ -19885,7 +19845,7 @@
         <v>894</v>
       </c>
       <c r="R18" s="3" t="s">
-        <v>1707</v>
+        <v>1692</v>
       </c>
       <c r="S18" s="3" t="s">
         <v>301</v>
@@ -19916,64 +19876,64 @@
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
+        <v>1693</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>1693</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>1694</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>1695</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>1696</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>1697</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>1698</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>1699</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>1700</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>1701</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>1702</v>
+      </c>
+      <c r="L19" s="3" t="s">
+        <v>1703</v>
+      </c>
+      <c r="M19" s="3" t="s">
+        <v>1704</v>
+      </c>
+      <c r="N19" s="3" t="s">
+        <v>1705</v>
+      </c>
+      <c r="O19" s="3" t="s">
+        <v>1706</v>
+      </c>
+      <c r="P19" s="3" t="s">
+        <v>1707</v>
+      </c>
+      <c r="Q19" s="3" t="s">
         <v>1708</v>
       </c>
-      <c r="B19" s="3" t="s">
-        <v>1708</v>
-      </c>
-      <c r="C19" s="3" t="s">
+      <c r="R19" s="3" t="s">
         <v>1709</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="S19" s="3" t="s">
         <v>1710</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="T19" s="3" t="s">
         <v>1711</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>1712</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>1713</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>1714</v>
-      </c>
-      <c r="I19" s="3" t="s">
-        <v>1715</v>
-      </c>
-      <c r="J19" s="3" t="s">
-        <v>1716</v>
-      </c>
-      <c r="K19" s="3" t="s">
-        <v>1717</v>
-      </c>
-      <c r="L19" s="3" t="s">
-        <v>1718</v>
-      </c>
-      <c r="M19" s="3" t="s">
-        <v>1719</v>
-      </c>
-      <c r="N19" s="3" t="s">
-        <v>1720</v>
-      </c>
-      <c r="O19" s="3" t="s">
-        <v>1721</v>
-      </c>
-      <c r="P19" s="3" t="s">
-        <v>1722</v>
-      </c>
-      <c r="Q19" s="3" t="s">
-        <v>1723</v>
-      </c>
-      <c r="R19" s="3" t="s">
-        <v>1724</v>
-      </c>
-      <c r="S19" s="3" t="s">
-        <v>1725</v>
-      </c>
-      <c r="T19" s="3" t="s">
-        <v>1726</v>
       </c>
       <c r="U19" s="4"/>
       <c r="V19" s="4"/>
@@ -19998,64 +19958,64 @@
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
+        <v>1712</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>1712</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>1713</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>1714</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>1715</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>1716</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>1717</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>1718</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>1719</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>1720</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>1721</v>
+      </c>
+      <c r="L20" s="3" t="s">
+        <v>1722</v>
+      </c>
+      <c r="M20" s="3" t="s">
+        <v>1723</v>
+      </c>
+      <c r="N20" s="3" t="s">
+        <v>1724</v>
+      </c>
+      <c r="O20" s="3" t="s">
+        <v>1725</v>
+      </c>
+      <c r="P20" s="3" t="s">
+        <v>1726</v>
+      </c>
+      <c r="Q20" s="3" t="s">
         <v>1727</v>
       </c>
-      <c r="B20" s="3" t="s">
-        <v>1727</v>
-      </c>
-      <c r="C20" s="3" t="s">
+      <c r="R20" s="3" t="s">
         <v>1728</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="S20" s="3" t="s">
         <v>1729</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="T20" s="3" t="s">
         <v>1730</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>1731</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>1732</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>1733</v>
-      </c>
-      <c r="I20" s="3" t="s">
-        <v>1734</v>
-      </c>
-      <c r="J20" s="3" t="s">
-        <v>1735</v>
-      </c>
-      <c r="K20" s="3" t="s">
-        <v>1736</v>
-      </c>
-      <c r="L20" s="3" t="s">
-        <v>1737</v>
-      </c>
-      <c r="M20" s="3" t="s">
-        <v>1738</v>
-      </c>
-      <c r="N20" s="3" t="s">
-        <v>1739</v>
-      </c>
-      <c r="O20" s="3" t="s">
-        <v>1740</v>
-      </c>
-      <c r="P20" s="3" t="s">
-        <v>1741</v>
-      </c>
-      <c r="Q20" s="3" t="s">
-        <v>1742</v>
-      </c>
-      <c r="R20" s="3" t="s">
-        <v>1743</v>
-      </c>
-      <c r="S20" s="3" t="s">
-        <v>1744</v>
-      </c>
-      <c r="T20" s="3" t="s">
-        <v>1745</v>
       </c>
       <c r="U20" s="4"/>
       <c r="V20" s="4"/>
@@ -20113,7 +20073,7 @@
         <v>331</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>1746</v>
+        <v>1731</v>
       </c>
       <c r="M21" s="3" t="s">
         <v>333</v>
@@ -20128,10 +20088,10 @@
         <v>336</v>
       </c>
       <c r="Q21" s="3" t="s">
-        <v>1747</v>
+        <v>1732</v>
       </c>
       <c r="R21" s="3" t="s">
-        <v>1748</v>
+        <v>1733</v>
       </c>
       <c r="S21" s="3" t="s">
         <v>339</v>
@@ -20241,7 +20201,7 @@
         <v>350</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>1749</v>
+        <v>1734</v>
       </c>
       <c r="M23" s="3" t="s">
         <v>352</v>
@@ -20259,7 +20219,7 @@
         <v>935</v>
       </c>
       <c r="R23" s="3" t="s">
-        <v>1750</v>
+        <v>1735</v>
       </c>
       <c r="S23" s="3" t="s">
         <v>358</v>
@@ -20323,7 +20283,7 @@
         <v>369</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>1751</v>
+        <v>1736</v>
       </c>
       <c r="M24" s="3" t="s">
         <v>371</v>
@@ -20341,7 +20301,7 @@
         <v>937</v>
       </c>
       <c r="R24" s="3" t="s">
-        <v>1752</v>
+        <v>1737</v>
       </c>
       <c r="S24" s="3" t="s">
         <v>377</v>
@@ -20405,7 +20365,7 @@
         <v>388</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>1753</v>
+        <v>1738</v>
       </c>
       <c r="M25" s="3" t="s">
         <v>390</v>
@@ -20423,7 +20383,7 @@
         <v>939</v>
       </c>
       <c r="R25" s="3" t="s">
-        <v>1754</v>
+        <v>1739</v>
       </c>
       <c r="S25" s="3" t="s">
         <v>396</v>
@@ -20487,7 +20447,7 @@
         <v>407</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>1755</v>
+        <v>1740</v>
       </c>
       <c r="M26" s="3" t="s">
         <v>409</v>
@@ -20505,7 +20465,7 @@
         <v>941</v>
       </c>
       <c r="R26" s="3" t="s">
-        <v>1756</v>
+        <v>1741</v>
       </c>
       <c r="S26" s="3" t="s">
         <v>415</v>
@@ -20569,7 +20529,7 @@
         <v>426</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>1757</v>
+        <v>1742</v>
       </c>
       <c r="M27" s="3" t="s">
         <v>428</v>
@@ -20584,10 +20544,10 @@
         <v>431</v>
       </c>
       <c r="Q27" s="3" t="s">
-        <v>1758</v>
+        <v>1743</v>
       </c>
       <c r="R27" s="3" t="s">
-        <v>1759</v>
+        <v>1744</v>
       </c>
       <c r="S27" s="3" t="s">
         <v>434</v>
@@ -20651,7 +20611,7 @@
         <v>445</v>
       </c>
       <c r="L28" s="3" t="s">
-        <v>1760</v>
+        <v>1745</v>
       </c>
       <c r="M28" s="3" t="s">
         <v>447</v>
@@ -20666,10 +20626,10 @@
         <v>450</v>
       </c>
       <c r="Q28" s="3" t="s">
-        <v>1761</v>
+        <v>1746</v>
       </c>
       <c r="R28" s="3" t="s">
-        <v>1762</v>
+        <v>1747</v>
       </c>
       <c r="S28" s="3" t="s">
         <v>453</v>
@@ -20733,7 +20693,7 @@
         <v>1522</v>
       </c>
       <c r="L29" s="3" t="s">
-        <v>1763</v>
+        <v>1748</v>
       </c>
       <c r="M29" s="3" t="s">
         <v>1524</v>
@@ -20742,7 +20702,7 @@
         <v>1525</v>
       </c>
       <c r="O29" s="3" t="s">
-        <v>1764</v>
+        <v>1749</v>
       </c>
       <c r="P29" s="3" t="s">
         <v>1527</v>
@@ -20815,7 +20775,7 @@
         <v>464</v>
       </c>
       <c r="L30" s="3" t="s">
-        <v>1765</v>
+        <v>1750</v>
       </c>
       <c r="M30" s="3" t="s">
         <v>466</v>
@@ -20833,7 +20793,7 @@
         <v>982</v>
       </c>
       <c r="R30" s="3" t="s">
-        <v>1766</v>
+        <v>1751</v>
       </c>
       <c r="S30" s="3" t="s">
         <v>472</v>
@@ -20897,7 +20857,7 @@
         <v>483</v>
       </c>
       <c r="L31" s="3" t="s">
-        <v>1767</v>
+        <v>1752</v>
       </c>
       <c r="M31" s="3" t="s">
         <v>485</v>
@@ -20915,7 +20875,7 @@
         <v>984</v>
       </c>
       <c r="R31" s="3" t="s">
-        <v>1768</v>
+        <v>1753</v>
       </c>
       <c r="S31" s="3" t="s">
         <v>491</v>
@@ -20979,7 +20939,7 @@
         <v>502</v>
       </c>
       <c r="L32" s="3" t="s">
-        <v>1769</v>
+        <v>1754</v>
       </c>
       <c r="M32" s="3" t="s">
         <v>504</v>
@@ -20997,7 +20957,7 @@
         <v>986</v>
       </c>
       <c r="R32" s="3" t="s">
-        <v>1770</v>
+        <v>1755</v>
       </c>
       <c r="S32" s="3" t="s">
         <v>510</v>
@@ -21061,7 +21021,7 @@
         <v>521</v>
       </c>
       <c r="L33" s="3" t="s">
-        <v>1771</v>
+        <v>1756</v>
       </c>
       <c r="M33" s="3" t="s">
         <v>523</v>
@@ -21076,10 +21036,10 @@
         <v>526</v>
       </c>
       <c r="Q33" s="3" t="s">
-        <v>1772</v>
+        <v>1757</v>
       </c>
       <c r="R33" s="3" t="s">
-        <v>1773</v>
+        <v>1758</v>
       </c>
       <c r="S33" s="3" t="s">
         <v>529</v>
@@ -21143,7 +21103,7 @@
         <v>540</v>
       </c>
       <c r="L34" s="3" t="s">
-        <v>1774</v>
+        <v>1759</v>
       </c>
       <c r="M34" s="3" t="s">
         <v>542</v>
@@ -21158,10 +21118,10 @@
         <v>545</v>
       </c>
       <c r="Q34" s="3" t="s">
-        <v>1775</v>
+        <v>1760</v>
       </c>
       <c r="R34" s="3" t="s">
-        <v>1776</v>
+        <v>1761</v>
       </c>
       <c r="S34" s="3" t="s">
         <v>548</v>
@@ -21192,64 +21152,64 @@
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
+        <v>1762</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>1762</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>1763</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>1764</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>1765</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>1766</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>1767</v>
+      </c>
+      <c r="H35" s="3" t="s">
+        <v>1768</v>
+      </c>
+      <c r="I35" s="3" t="s">
+        <v>1769</v>
+      </c>
+      <c r="J35" s="3" t="s">
+        <v>1770</v>
+      </c>
+      <c r="K35" s="3" t="s">
+        <v>1771</v>
+      </c>
+      <c r="L35" s="3" t="s">
+        <v>1772</v>
+      </c>
+      <c r="M35" s="3" t="s">
+        <v>1773</v>
+      </c>
+      <c r="N35" s="3" t="s">
+        <v>1774</v>
+      </c>
+      <c r="O35" s="3" t="s">
+        <v>1775</v>
+      </c>
+      <c r="P35" s="3" t="s">
+        <v>1776</v>
+      </c>
+      <c r="Q35" s="3" t="s">
         <v>1777</v>
       </c>
-      <c r="B35" s="3" t="s">
-        <v>1777</v>
-      </c>
-      <c r="C35" s="3" t="s">
+      <c r="R35" s="3" t="s">
         <v>1778</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="S35" s="3" t="s">
         <v>1779</v>
       </c>
-      <c r="E35" s="3" t="s">
+      <c r="T35" s="3" t="s">
         <v>1780</v>
-      </c>
-      <c r="F35" s="3" t="s">
-        <v>1781</v>
-      </c>
-      <c r="G35" s="3" t="s">
-        <v>1782</v>
-      </c>
-      <c r="H35" s="3" t="s">
-        <v>1783</v>
-      </c>
-      <c r="I35" s="3" t="s">
-        <v>1784</v>
-      </c>
-      <c r="J35" s="3" t="s">
-        <v>1785</v>
-      </c>
-      <c r="K35" s="3" t="s">
-        <v>1786</v>
-      </c>
-      <c r="L35" s="3" t="s">
-        <v>1787</v>
-      </c>
-      <c r="M35" s="3" t="s">
-        <v>1788</v>
-      </c>
-      <c r="N35" s="3" t="s">
-        <v>1789</v>
-      </c>
-      <c r="O35" s="3" t="s">
-        <v>1790</v>
-      </c>
-      <c r="P35" s="3" t="s">
-        <v>1791</v>
-      </c>
-      <c r="Q35" s="3" t="s">
-        <v>1792</v>
-      </c>
-      <c r="R35" s="3" t="s">
-        <v>1793</v>
-      </c>
-      <c r="S35" s="3" t="s">
-        <v>1794</v>
-      </c>
-      <c r="T35" s="3" t="s">
-        <v>1795</v>
       </c>
       <c r="U35" s="4"/>
       <c r="V35" s="4"/>
@@ -21274,64 +21234,64 @@
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
+        <v>1781</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>1781</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>1782</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>1783</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>1784</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>1785</v>
+      </c>
+      <c r="G36" s="3" t="s">
+        <v>1786</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>1787</v>
+      </c>
+      <c r="I36" s="3" t="s">
+        <v>1788</v>
+      </c>
+      <c r="J36" s="3" t="s">
+        <v>1789</v>
+      </c>
+      <c r="K36" s="3" t="s">
+        <v>1790</v>
+      </c>
+      <c r="L36" s="3" t="s">
+        <v>1791</v>
+      </c>
+      <c r="M36" s="3" t="s">
+        <v>1792</v>
+      </c>
+      <c r="N36" s="3" t="s">
+        <v>1793</v>
+      </c>
+      <c r="O36" s="3" t="s">
+        <v>1794</v>
+      </c>
+      <c r="P36" s="3" t="s">
+        <v>1795</v>
+      </c>
+      <c r="Q36" s="3" t="s">
         <v>1796</v>
       </c>
-      <c r="B36" s="3" t="s">
-        <v>1796</v>
-      </c>
-      <c r="C36" s="3" t="s">
+      <c r="R36" s="3" t="s">
         <v>1797</v>
       </c>
-      <c r="D36" s="3" t="s">
+      <c r="S36" s="3" t="s">
         <v>1798</v>
       </c>
-      <c r="E36" s="3" t="s">
+      <c r="T36" s="3" t="s">
         <v>1799</v>
-      </c>
-      <c r="F36" s="3" t="s">
-        <v>1800</v>
-      </c>
-      <c r="G36" s="3" t="s">
-        <v>1801</v>
-      </c>
-      <c r="H36" s="3" t="s">
-        <v>1802</v>
-      </c>
-      <c r="I36" s="3" t="s">
-        <v>1803</v>
-      </c>
-      <c r="J36" s="3" t="s">
-        <v>1804</v>
-      </c>
-      <c r="K36" s="3" t="s">
-        <v>1805</v>
-      </c>
-      <c r="L36" s="3" t="s">
-        <v>1806</v>
-      </c>
-      <c r="M36" s="3" t="s">
-        <v>1807</v>
-      </c>
-      <c r="N36" s="3" t="s">
-        <v>1808</v>
-      </c>
-      <c r="O36" s="3" t="s">
-        <v>1809</v>
-      </c>
-      <c r="P36" s="3" t="s">
-        <v>1810</v>
-      </c>
-      <c r="Q36" s="3" t="s">
-        <v>1811</v>
-      </c>
-      <c r="R36" s="3" t="s">
-        <v>1812</v>
-      </c>
-      <c r="S36" s="3" t="s">
-        <v>1813</v>
-      </c>
-      <c r="T36" s="3" t="s">
-        <v>1814</v>
       </c>
       <c r="U36" s="4"/>
       <c r="V36" s="4"/>
@@ -21389,7 +21349,7 @@
         <v>274</v>
       </c>
       <c r="L37" s="3" t="s">
-        <v>1815</v>
+        <v>1800</v>
       </c>
       <c r="M37" s="3" t="s">
         <v>276</v>
@@ -21407,7 +21367,7 @@
         <v>892</v>
       </c>
       <c r="R37" s="3" t="s">
-        <v>1816</v>
+        <v>1801</v>
       </c>
       <c r="S37" s="3" t="s">
         <v>282</v>
@@ -21438,64 +21398,64 @@
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
+        <v>1802</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>1802</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>1803</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>1804</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>1805</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>1806</v>
+      </c>
+      <c r="G38" s="3" t="s">
+        <v>1807</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>1808</v>
+      </c>
+      <c r="I38" s="3" t="s">
+        <v>1809</v>
+      </c>
+      <c r="J38" s="3" t="s">
+        <v>1810</v>
+      </c>
+      <c r="K38" s="3" t="s">
+        <v>1811</v>
+      </c>
+      <c r="L38" s="3" t="s">
+        <v>1812</v>
+      </c>
+      <c r="M38" s="3" t="s">
+        <v>1813</v>
+      </c>
+      <c r="N38" s="3" t="s">
+        <v>1814</v>
+      </c>
+      <c r="O38" s="3" t="s">
+        <v>1815</v>
+      </c>
+      <c r="P38" s="3" t="s">
+        <v>1816</v>
+      </c>
+      <c r="Q38" s="3" t="s">
         <v>1817</v>
       </c>
-      <c r="B38" s="3" t="s">
-        <v>1817</v>
-      </c>
-      <c r="C38" s="3" t="s">
+      <c r="R38" s="3" t="s">
         <v>1818</v>
       </c>
-      <c r="D38" s="3" t="s">
+      <c r="S38" s="3" t="s">
         <v>1819</v>
       </c>
-      <c r="E38" s="3" t="s">
+      <c r="T38" s="3" t="s">
         <v>1820</v>
-      </c>
-      <c r="F38" s="3" t="s">
-        <v>1821</v>
-      </c>
-      <c r="G38" s="3" t="s">
-        <v>1822</v>
-      </c>
-      <c r="H38" s="3" t="s">
-        <v>1823</v>
-      </c>
-      <c r="I38" s="3" t="s">
-        <v>1824</v>
-      </c>
-      <c r="J38" s="3" t="s">
-        <v>1825</v>
-      </c>
-      <c r="K38" s="3" t="s">
-        <v>1826</v>
-      </c>
-      <c r="L38" s="3" t="s">
-        <v>1827</v>
-      </c>
-      <c r="M38" s="3" t="s">
-        <v>1828</v>
-      </c>
-      <c r="N38" s="3" t="s">
-        <v>1829</v>
-      </c>
-      <c r="O38" s="3" t="s">
-        <v>1830</v>
-      </c>
-      <c r="P38" s="3" t="s">
-        <v>1831</v>
-      </c>
-      <c r="Q38" s="3" t="s">
-        <v>1832</v>
-      </c>
-      <c r="R38" s="3" t="s">
-        <v>1833</v>
-      </c>
-      <c r="S38" s="3" t="s">
-        <v>1834</v>
-      </c>
-      <c r="T38" s="3" t="s">
-        <v>1835</v>
       </c>
       <c r="U38" s="4"/>
       <c r="V38" s="4"/>
@@ -21553,7 +21513,7 @@
         <v>312</v>
       </c>
       <c r="L39" s="3" t="s">
-        <v>1836</v>
+        <v>1821</v>
       </c>
       <c r="M39" s="3" t="s">
         <v>314</v>
@@ -21568,10 +21528,10 @@
         <v>317</v>
       </c>
       <c r="Q39" s="3" t="s">
-        <v>1837</v>
+        <v>1822</v>
       </c>
       <c r="R39" s="3" t="s">
-        <v>1838</v>
+        <v>1823</v>
       </c>
       <c r="S39" s="3" t="s">
         <v>320</v>
@@ -21602,64 +21562,64 @@
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
+        <v>1824</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>1824</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>1825</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>1826</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>1827</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>1828</v>
+      </c>
+      <c r="G40" s="3" t="s">
+        <v>1829</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>1830</v>
+      </c>
+      <c r="I40" s="3" t="s">
+        <v>1831</v>
+      </c>
+      <c r="J40" s="3" t="s">
+        <v>1832</v>
+      </c>
+      <c r="K40" s="3" t="s">
+        <v>1833</v>
+      </c>
+      <c r="L40" s="3" t="s">
+        <v>1834</v>
+      </c>
+      <c r="M40" s="3" t="s">
+        <v>1835</v>
+      </c>
+      <c r="N40" s="3" t="s">
+        <v>1836</v>
+      </c>
+      <c r="O40" s="3" t="s">
+        <v>1837</v>
+      </c>
+      <c r="P40" s="3" t="s">
+        <v>1838</v>
+      </c>
+      <c r="Q40" s="3" t="s">
         <v>1839</v>
       </c>
-      <c r="B40" s="3" t="s">
-        <v>1839</v>
-      </c>
-      <c r="C40" s="3" t="s">
+      <c r="R40" s="3" t="s">
         <v>1840</v>
       </c>
-      <c r="D40" s="3" t="s">
+      <c r="S40" s="3" t="s">
         <v>1841</v>
       </c>
-      <c r="E40" s="3" t="s">
+      <c r="T40" s="3" t="s">
         <v>1842</v>
-      </c>
-      <c r="F40" s="3" t="s">
-        <v>1843</v>
-      </c>
-      <c r="G40" s="3" t="s">
-        <v>1844</v>
-      </c>
-      <c r="H40" s="3" t="s">
-        <v>1845</v>
-      </c>
-      <c r="I40" s="3" t="s">
-        <v>1846</v>
-      </c>
-      <c r="J40" s="3" t="s">
-        <v>1847</v>
-      </c>
-      <c r="K40" s="3" t="s">
-        <v>1848</v>
-      </c>
-      <c r="L40" s="3" t="s">
-        <v>1849</v>
-      </c>
-      <c r="M40" s="3" t="s">
-        <v>1850</v>
-      </c>
-      <c r="N40" s="3" t="s">
-        <v>1851</v>
-      </c>
-      <c r="O40" s="3" t="s">
-        <v>1852</v>
-      </c>
-      <c r="P40" s="3" t="s">
-        <v>1853</v>
-      </c>
-      <c r="Q40" s="3" t="s">
-        <v>1854</v>
-      </c>
-      <c r="R40" s="3" t="s">
-        <v>1855</v>
-      </c>
-      <c r="S40" s="3" t="s">
-        <v>1856</v>
-      </c>
-      <c r="T40" s="3" t="s">
-        <v>1857</v>
       </c>
       <c r="U40" s="4"/>
       <c r="V40" s="4"/>
@@ -21717,7 +21677,7 @@
         <v>673</v>
       </c>
       <c r="L41" s="3" t="s">
-        <v>1858</v>
+        <v>1843</v>
       </c>
       <c r="M41" s="3" t="s">
         <v>675</v>
@@ -21735,7 +21695,7 @@
         <v>1140</v>
       </c>
       <c r="R41" s="3" t="s">
-        <v>1859</v>
+        <v>1844</v>
       </c>
       <c r="S41" s="3" t="s">
         <v>681</v>
@@ -21799,7 +21759,7 @@
         <v>692</v>
       </c>
       <c r="L42" s="3" t="s">
-        <v>1860</v>
+        <v>1845</v>
       </c>
       <c r="M42" s="3" t="s">
         <v>694</v>
@@ -21817,7 +21777,7 @@
         <v>1142</v>
       </c>
       <c r="R42" s="3" t="s">
-        <v>1861</v>
+        <v>1846</v>
       </c>
       <c r="S42" s="3" t="s">
         <v>700</v>
@@ -21881,7 +21841,7 @@
         <v>350</v>
       </c>
       <c r="L43" s="3" t="s">
-        <v>1749</v>
+        <v>1734</v>
       </c>
       <c r="M43" s="3" t="s">
         <v>352</v>
@@ -21899,7 +21859,7 @@
         <v>935</v>
       </c>
       <c r="R43" s="3" t="s">
-        <v>1750</v>
+        <v>1735</v>
       </c>
       <c r="S43" s="3" t="s">
         <v>358</v>
@@ -21963,7 +21923,7 @@
         <v>730</v>
       </c>
       <c r="L44" s="3" t="s">
-        <v>1862</v>
+        <v>1847</v>
       </c>
       <c r="M44" s="3" t="s">
         <v>732</v>
@@ -21981,7 +21941,7 @@
         <v>1146</v>
       </c>
       <c r="R44" s="3" t="s">
-        <v>1863</v>
+        <v>1848</v>
       </c>
       <c r="S44" s="3" t="s">
         <v>738</v>
@@ -22045,7 +22005,7 @@
         <v>749</v>
       </c>
       <c r="L45" s="3" t="s">
-        <v>1864</v>
+        <v>1849</v>
       </c>
       <c r="M45" s="3" t="s">
         <v>751</v>
@@ -22063,7 +22023,7 @@
         <v>1148</v>
       </c>
       <c r="R45" s="3" t="s">
-        <v>1865</v>
+        <v>1850</v>
       </c>
       <c r="S45" s="3" t="s">
         <v>757</v>
@@ -22127,7 +22087,7 @@
         <v>768</v>
       </c>
       <c r="L46" s="3" t="s">
-        <v>1866</v>
+        <v>1851</v>
       </c>
       <c r="M46" s="3" t="s">
         <v>770</v>
@@ -22142,10 +22102,10 @@
         <v>773</v>
       </c>
       <c r="Q46" s="3" t="s">
-        <v>1867</v>
+        <v>1852</v>
       </c>
       <c r="R46" s="3" t="s">
-        <v>1868</v>
+        <v>1853</v>
       </c>
       <c r="S46" s="3" t="s">
         <v>776</v>
@@ -22209,7 +22169,7 @@
         <v>787</v>
       </c>
       <c r="L47" s="3" t="s">
-        <v>1869</v>
+        <v>1854</v>
       </c>
       <c r="M47" s="3" t="s">
         <v>789</v>
@@ -22224,10 +22184,10 @@
         <v>792</v>
       </c>
       <c r="Q47" s="3" t="s">
-        <v>1870</v>
+        <v>1855</v>
       </c>
       <c r="R47" s="3" t="s">
-        <v>1871</v>
+        <v>1856</v>
       </c>
       <c r="S47" s="3" t="s">
         <v>795</v>
@@ -22273,10 +22233,10 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AN47"/>
-  <sheetFormatPr defaultColWidth="14.5078125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.515625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="1" style="1" width="8.68"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="41" style="1" width="14.51"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="41" style="1" width="14.52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22327,13 +22287,13 @@
         <v>14</v>
       </c>
       <c r="Q1" s="3" t="s">
-        <v>1872</v>
+        <v>1857</v>
       </c>
       <c r="R1" s="3" t="s">
-        <v>1873</v>
+        <v>1858</v>
       </c>
       <c r="S1" s="3" t="s">
-        <v>1874</v>
+        <v>1859</v>
       </c>
       <c r="T1" s="3" t="s">
         <v>18</v>
@@ -22445,7 +22405,7 @@
         <v>51</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>1875</v>
+        <v>1860</v>
       </c>
       <c r="R2" s="3" t="s">
         <v>800</v>
@@ -22458,44 +22418,44 @@
       </c>
       <c r="U2" s="4"/>
       <c r="V2" s="3" t="s">
-        <v>1876</v>
+        <v>1861</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>1877</v>
+        <v>1862</v>
       </c>
       <c r="X2" s="3" t="s">
-        <v>1878</v>
+        <v>1863</v>
       </c>
       <c r="Y2" s="3" t="s">
-        <v>1879</v>
+        <v>1864</v>
       </c>
       <c r="Z2" s="5" t="s">
-        <v>1880</v>
+        <v>1865</v>
       </c>
       <c r="AA2" s="3" t="s">
-        <v>1881</v>
+        <v>1866</v>
       </c>
       <c r="AB2" s="3" t="s">
-        <v>1882</v>
+        <v>1867</v>
       </c>
       <c r="AC2" s="3" t="s">
-        <v>1883</v>
+        <v>1868</v>
       </c>
       <c r="AD2" s="5" t="s">
-        <v>1884</v>
+        <v>1869</v>
       </c>
       <c r="AE2" s="3"/>
       <c r="AF2" s="3" t="s">
-        <v>1885</v>
+        <v>1870</v>
       </c>
       <c r="AG2" s="3" t="s">
-        <v>1886</v>
+        <v>1871</v>
       </c>
       <c r="AH2" s="3" t="s">
-        <v>1886</v>
+        <v>1871</v>
       </c>
       <c r="AI2" s="3" t="s">
-        <v>1876</v>
+        <v>1861</v>
       </c>
       <c r="AJ2" s="4" t="n">
         <v>321</v>
@@ -22504,13 +22464,13 @@
         <v>521</v>
       </c>
       <c r="AL2" s="3" t="s">
-        <v>1887</v>
+        <v>1872</v>
       </c>
       <c r="AM2" s="3" t="s">
-        <v>1879</v>
+        <v>1864</v>
       </c>
       <c r="AN2" s="3" t="s">
-        <v>1877</v>
+        <v>1862</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22563,7 +22523,7 @@
         <v>70</v>
       </c>
       <c r="Q3" s="3" t="s">
-        <v>1888</v>
+        <v>1873</v>
       </c>
       <c r="R3" s="3" t="s">
         <v>802</v>
@@ -22645,7 +22605,7 @@
         <v>817</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>1889</v>
+        <v>1874</v>
       </c>
       <c r="R4" s="3" t="s">
         <v>819</v>
@@ -22727,7 +22687,7 @@
         <v>817</v>
       </c>
       <c r="Q5" s="3" t="s">
-        <v>1889</v>
+        <v>1874</v>
       </c>
       <c r="R5" s="3" t="s">
         <v>819</v>
@@ -22809,7 +22769,7 @@
         <v>108</v>
       </c>
       <c r="Q6" s="3" t="s">
-        <v>1890</v>
+        <v>1875</v>
       </c>
       <c r="R6" s="3" t="s">
         <v>823</v>
@@ -22891,7 +22851,7 @@
         <v>127</v>
       </c>
       <c r="Q7" s="3" t="s">
-        <v>1891</v>
+        <v>1876</v>
       </c>
       <c r="R7" s="3" t="s">
         <v>825</v>
@@ -22973,7 +22933,7 @@
         <v>146</v>
       </c>
       <c r="Q8" s="3" t="s">
-        <v>1892</v>
+        <v>1877</v>
       </c>
       <c r="R8" s="3" t="s">
         <v>827</v>
@@ -23055,7 +23015,7 @@
         <v>842</v>
       </c>
       <c r="Q9" s="3" t="s">
-        <v>1893</v>
+        <v>1878</v>
       </c>
       <c r="R9" s="3" t="s">
         <v>844</v>
@@ -23137,7 +23097,7 @@
         <v>861</v>
       </c>
       <c r="Q10" s="3" t="s">
-        <v>1894</v>
+        <v>1879</v>
       </c>
       <c r="R10" s="3" t="s">
         <v>863</v>
@@ -23219,7 +23179,7 @@
         <v>880</v>
       </c>
       <c r="Q11" s="3" t="s">
-        <v>1895</v>
+        <v>1880</v>
       </c>
       <c r="R11" s="3" t="s">
         <v>882</v>
@@ -23347,7 +23307,7 @@
         <v>222</v>
       </c>
       <c r="Q13" s="3" t="s">
-        <v>1896</v>
+        <v>1881</v>
       </c>
       <c r="R13" s="3" t="s">
         <v>886</v>
@@ -23432,10 +23392,10 @@
         <v>887</v>
       </c>
       <c r="R14" s="3" t="s">
-        <v>1897</v>
+        <v>1882</v>
       </c>
       <c r="S14" s="3" t="s">
-        <v>1763</v>
+        <v>1748</v>
       </c>
       <c r="T14" s="3" t="s">
         <v>245</v>
@@ -23513,7 +23473,7 @@
         <v>260</v>
       </c>
       <c r="Q15" s="3" t="s">
-        <v>1898</v>
+        <v>1883</v>
       </c>
       <c r="R15" s="3" t="s">
         <v>891</v>
@@ -23595,7 +23555,7 @@
         <v>279</v>
       </c>
       <c r="Q16" s="3" t="s">
-        <v>1899</v>
+        <v>1884</v>
       </c>
       <c r="R16" s="3" t="s">
         <v>893</v>
@@ -23677,7 +23637,7 @@
         <v>298</v>
       </c>
       <c r="Q17" s="3" t="s">
-        <v>1900</v>
+        <v>1885</v>
       </c>
       <c r="R17" s="3" t="s">
         <v>895</v>
@@ -23759,7 +23719,7 @@
         <v>298</v>
       </c>
       <c r="Q18" s="3" t="s">
-        <v>1900</v>
+        <v>1885</v>
       </c>
       <c r="R18" s="3" t="s">
         <v>895</v>
@@ -23841,7 +23801,7 @@
         <v>910</v>
       </c>
       <c r="Q19" s="3" t="s">
-        <v>1901</v>
+        <v>1886</v>
       </c>
       <c r="R19" s="3" t="s">
         <v>912</v>
@@ -23923,7 +23883,7 @@
         <v>929</v>
       </c>
       <c r="Q20" s="3" t="s">
-        <v>1902</v>
+        <v>1887</v>
       </c>
       <c r="R20" s="3" t="s">
         <v>931</v>
@@ -24005,7 +23965,7 @@
         <v>929</v>
       </c>
       <c r="Q21" s="3" t="s">
-        <v>1902</v>
+        <v>1887</v>
       </c>
       <c r="R21" s="3" t="s">
         <v>931</v>
@@ -24133,7 +24093,7 @@
         <v>355</v>
       </c>
       <c r="Q23" s="3" t="s">
-        <v>1903</v>
+        <v>1888</v>
       </c>
       <c r="R23" s="3" t="s">
         <v>936</v>
@@ -24215,7 +24175,7 @@
         <v>374</v>
       </c>
       <c r="Q24" s="3" t="s">
-        <v>1904</v>
+        <v>1889</v>
       </c>
       <c r="R24" s="3" t="s">
         <v>938</v>
@@ -24297,7 +24257,7 @@
         <v>393</v>
       </c>
       <c r="Q25" s="3" t="s">
-        <v>1905</v>
+        <v>1890</v>
       </c>
       <c r="R25" s="3" t="s">
         <v>940</v>
@@ -24379,7 +24339,7 @@
         <v>412</v>
       </c>
       <c r="Q26" s="3" t="s">
-        <v>1906</v>
+        <v>1891</v>
       </c>
       <c r="R26" s="3" t="s">
         <v>942</v>
@@ -24461,7 +24421,7 @@
         <v>957</v>
       </c>
       <c r="Q27" s="3" t="s">
-        <v>1907</v>
+        <v>1892</v>
       </c>
       <c r="R27" s="3" t="s">
         <v>959</v>
@@ -24543,7 +24503,7 @@
         <v>976</v>
       </c>
       <c r="Q28" s="3" t="s">
-        <v>1908</v>
+        <v>1893</v>
       </c>
       <c r="R28" s="3" t="s">
         <v>978</v>
@@ -24628,10 +24588,10 @@
         <v>887</v>
       </c>
       <c r="R29" s="3" t="s">
-        <v>1897</v>
+        <v>1882</v>
       </c>
       <c r="S29" s="3" t="s">
-        <v>1763</v>
+        <v>1748</v>
       </c>
       <c r="T29" s="3" t="s">
         <v>245</v>
@@ -24710,10 +24670,10 @@
         <v>982</v>
       </c>
       <c r="R30" s="3" t="s">
-        <v>1909</v>
+        <v>1894</v>
       </c>
       <c r="S30" s="3" t="s">
-        <v>1765</v>
+        <v>1750</v>
       </c>
       <c r="T30" s="3" t="s">
         <v>473</v>
@@ -24792,10 +24752,10 @@
         <v>984</v>
       </c>
       <c r="R31" s="3" t="s">
-        <v>1910</v>
+        <v>1895</v>
       </c>
       <c r="S31" s="3" t="s">
-        <v>1767</v>
+        <v>1752</v>
       </c>
       <c r="T31" s="3" t="s">
         <v>492</v>
@@ -24874,10 +24834,10 @@
         <v>986</v>
       </c>
       <c r="R32" s="3" t="s">
-        <v>1911</v>
+        <v>1896</v>
       </c>
       <c r="S32" s="3" t="s">
-        <v>1769</v>
+        <v>1754</v>
       </c>
       <c r="T32" s="3" t="s">
         <v>511</v>
@@ -24956,10 +24916,10 @@
         <v>1003</v>
       </c>
       <c r="R33" s="3" t="s">
-        <v>1912</v>
+        <v>1897</v>
       </c>
       <c r="S33" s="3" t="s">
-        <v>1913</v>
+        <v>1898</v>
       </c>
       <c r="T33" s="3" t="s">
         <v>1006</v>
@@ -25038,10 +24998,10 @@
         <v>1022</v>
       </c>
       <c r="R34" s="3" t="s">
-        <v>1914</v>
+        <v>1899</v>
       </c>
       <c r="S34" s="3" t="s">
-        <v>1915</v>
+        <v>1900</v>
       </c>
       <c r="T34" s="3" t="s">
         <v>1025</v>
@@ -25120,10 +25080,10 @@
         <v>1041</v>
       </c>
       <c r="R35" s="3" t="s">
-        <v>1916</v>
+        <v>1901</v>
       </c>
       <c r="S35" s="3" t="s">
-        <v>1917</v>
+        <v>1902</v>
       </c>
       <c r="T35" s="3" t="s">
         <v>1044</v>
@@ -25202,10 +25162,10 @@
         <v>1060</v>
       </c>
       <c r="R36" s="3" t="s">
-        <v>1918</v>
+        <v>1903</v>
       </c>
       <c r="S36" s="3" t="s">
-        <v>1919</v>
+        <v>1904</v>
       </c>
       <c r="T36" s="3" t="s">
         <v>1063</v>
@@ -25284,10 +25244,10 @@
         <v>1079</v>
       </c>
       <c r="R37" s="3" t="s">
-        <v>1920</v>
+        <v>1905</v>
       </c>
       <c r="S37" s="3" t="s">
-        <v>1921</v>
+        <v>1906</v>
       </c>
       <c r="T37" s="3" t="s">
         <v>1082</v>
@@ -25366,10 +25326,10 @@
         <v>1098</v>
       </c>
       <c r="R38" s="3" t="s">
-        <v>1922</v>
+        <v>1907</v>
       </c>
       <c r="S38" s="3" t="s">
-        <v>1923</v>
+        <v>1908</v>
       </c>
       <c r="T38" s="3" t="s">
         <v>1101</v>
@@ -25448,10 +25408,10 @@
         <v>1117</v>
       </c>
       <c r="R39" s="3" t="s">
-        <v>1924</v>
+        <v>1909</v>
       </c>
       <c r="S39" s="3" t="s">
-        <v>1925</v>
+        <v>1910</v>
       </c>
       <c r="T39" s="3" t="s">
         <v>1120</v>
@@ -25530,10 +25490,10 @@
         <v>1136</v>
       </c>
       <c r="R40" s="3" t="s">
-        <v>1926</v>
+        <v>1911</v>
       </c>
       <c r="S40" s="3" t="s">
-        <v>1927</v>
+        <v>1912</v>
       </c>
       <c r="T40" s="3" t="s">
         <v>1139</v>
@@ -25609,7 +25569,7 @@
         <v>678</v>
       </c>
       <c r="Q41" s="3" t="s">
-        <v>1928</v>
+        <v>1913</v>
       </c>
       <c r="R41" s="3" t="s">
         <v>1141</v>
@@ -25691,7 +25651,7 @@
         <v>697</v>
       </c>
       <c r="Q42" s="3" t="s">
-        <v>1929</v>
+        <v>1914</v>
       </c>
       <c r="R42" s="3" t="s">
         <v>1143</v>
@@ -25773,7 +25733,7 @@
         <v>716</v>
       </c>
       <c r="Q43" s="3" t="s">
-        <v>1930</v>
+        <v>1915</v>
       </c>
       <c r="R43" s="3" t="s">
         <v>1145</v>
@@ -25855,7 +25815,7 @@
         <v>735</v>
       </c>
       <c r="Q44" s="3" t="s">
-        <v>1931</v>
+        <v>1916</v>
       </c>
       <c r="R44" s="3" t="s">
         <v>1147</v>
@@ -25937,7 +25897,7 @@
         <v>754</v>
       </c>
       <c r="Q45" s="3" t="s">
-        <v>1932</v>
+        <v>1917</v>
       </c>
       <c r="R45" s="3" t="s">
         <v>1149</v>
@@ -26019,7 +25979,7 @@
         <v>1164</v>
       </c>
       <c r="Q46" s="3" t="s">
-        <v>1933</v>
+        <v>1918</v>
       </c>
       <c r="R46" s="3" t="s">
         <v>1166</v>
@@ -26101,7 +26061,7 @@
         <v>1183</v>
       </c>
       <c r="Q47" s="3" t="s">
-        <v>1934</v>
+        <v>1919</v>
       </c>
       <c r="R47" s="3" t="s">
         <v>1185</v>
@@ -26150,7 +26110,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I15"/>
-  <sheetFormatPr defaultColWidth="14.5078125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.515625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="36.35"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10"/>
@@ -26161,19 +26121,19 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="12.68"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="8.68"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="10" style="1" width="14.51"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="10" style="1" width="14.52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>1935</v>
+        <v>1920</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
       <c r="D1" s="6"/>
       <c r="E1" s="7"/>
       <c r="F1" s="6" t="s">
-        <v>1936</v>
+        <v>1921</v>
       </c>
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
@@ -26181,34 +26141,34 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>1937</v>
+        <v>1922</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>1938</v>
+        <v>1923</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>1939</v>
+        <v>1924</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>1940</v>
+        <v>1925</v>
       </c>
       <c r="E2" s="7"/>
       <c r="F2" s="8" t="s">
-        <v>1937</v>
+        <v>1922</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>1938</v>
+        <v>1923</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>1939</v>
+        <v>1924</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>1940</v>
+        <v>1925</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>1941</v>
+        <v>1926</v>
       </c>
       <c r="B3" s="11" t="s">
         <v>6</v>
@@ -26221,7 +26181,7 @@
       </c>
       <c r="E3" s="7"/>
       <c r="F3" s="8" t="s">
-        <v>1942</v>
+        <v>1927</v>
       </c>
       <c r="G3" s="11" t="s">
         <v>14</v>
@@ -26235,110 +26195,110 @@
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>1943</v>
+        <v>1928</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="E4" s="7"/>
       <c r="F4" s="8" t="s">
-        <v>1945</v>
+        <v>1930</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="I4" s="14" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>1946</v>
+        <v>1931</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="E5" s="7"/>
       <c r="F5" s="8" t="s">
-        <v>1946</v>
+        <v>1931</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="H5" s="12" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="I5" s="14" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>1947</v>
+        <v>1932</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="E6" s="7"/>
       <c r="F6" s="8" t="s">
-        <v>1947</v>
+        <v>1932</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="H6" s="12" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="I6" s="14" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>1948</v>
+        <v>1933</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="E7" s="7"/>
       <c r="F7" s="15" t="s">
-        <v>1948</v>
+        <v>1933</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="H7" s="17" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="I7" s="18" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26354,14 +26314,14 @@
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>1935</v>
+        <v>1920</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
       <c r="D9" s="6"/>
       <c r="E9" s="7"/>
       <c r="F9" s="6" t="s">
-        <v>1936</v>
+        <v>1921</v>
       </c>
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>
@@ -26369,30 +26329,30 @@
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>1937</v>
+        <v>1922</v>
       </c>
       <c r="B10" s="20"/>
       <c r="C10" s="9" t="s">
-        <v>1949</v>
+        <v>1934</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>1940</v>
+        <v>1925</v>
       </c>
       <c r="E10" s="7"/>
       <c r="F10" s="20" t="s">
-        <v>1937</v>
+        <v>1922</v>
       </c>
       <c r="G10" s="20"/>
       <c r="H10" s="9" t="s">
-        <v>1949</v>
+        <v>1934</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>1940</v>
+        <v>1925</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>1941</v>
+        <v>1926</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="21" t="s">
@@ -26403,7 +26363,7 @@
       </c>
       <c r="E11" s="7"/>
       <c r="F11" s="20" t="s">
-        <v>1942</v>
+        <v>1927</v>
       </c>
       <c r="G11" s="20"/>
       <c r="H11" s="21" t="s">
@@ -26415,94 +26375,94 @@
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>1943</v>
+        <v>1928</v>
       </c>
       <c r="B12" s="20"/>
       <c r="C12" s="21" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="E12" s="7"/>
       <c r="F12" s="20" t="s">
-        <v>1945</v>
+        <v>1930</v>
       </c>
       <c r="G12" s="20"/>
       <c r="H12" s="21" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="I12" s="14" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>1946</v>
+        <v>1931</v>
       </c>
       <c r="B13" s="20"/>
       <c r="C13" s="21" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="E13" s="7"/>
       <c r="F13" s="20" t="s">
-        <v>1946</v>
+        <v>1931</v>
       </c>
       <c r="G13" s="20"/>
       <c r="H13" s="21" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="I13" s="14" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>1947</v>
+        <v>1932</v>
       </c>
       <c r="B14" s="20"/>
       <c r="C14" s="21" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="E14" s="7"/>
       <c r="F14" s="20" t="s">
-        <v>1947</v>
+        <v>1932</v>
       </c>
       <c r="G14" s="20"/>
       <c r="H14" s="21" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="I14" s="14" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="22" t="s">
-        <v>1948</v>
+        <v>1933</v>
       </c>
       <c r="B15" s="22"/>
       <c r="C15" s="23" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="E15" s="7"/>
       <c r="F15" s="22" t="s">
-        <v>1948</v>
+        <v>1933</v>
       </c>
       <c r="G15" s="22"/>
       <c r="H15" s="23" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
       <c r="I15" s="18" t="s">
-        <v>1944</v>
+        <v>1929</v>
       </c>
     </row>
   </sheetData>
@@ -26540,20 +26500,20 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E40"/>
-  <sheetFormatPr defaultColWidth="14.5078125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.515625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.35"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="51.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="38.35"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="32.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="29.35"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16383" min="7" style="1" width="14.51"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16383" min="7" style="1" width="14.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="24" t="s">
-        <v>1950</v>
+        <v>1935</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -26562,169 +26522,169 @@
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="25" t="s">
-        <v>1951</v>
+        <v>1936</v>
       </c>
       <c r="B2" s="25"/>
       <c r="C2" s="25"/>
       <c r="D2" s="26"/>
       <c r="E2" s="27" t="s">
-        <v>1952</v>
+        <v>1937</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="28" t="s">
-        <v>1953</v>
+        <v>1938</v>
       </c>
       <c r="B3" s="28" t="s">
-        <v>1954</v>
+        <v>1939</v>
       </c>
       <c r="C3" s="28" t="s">
-        <v>1955</v>
+        <v>1940</v>
       </c>
       <c r="D3" s="28" t="s">
-        <v>1956</v>
+        <v>1941</v>
       </c>
       <c r="E3" s="27"/>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="29" t="s">
-        <v>1957</v>
+        <v>1942</v>
       </c>
       <c r="B4" s="29" t="s">
-        <v>1958</v>
+        <v>1943</v>
       </c>
       <c r="C4" s="29" t="s">
-        <v>1959</v>
+        <v>1944</v>
       </c>
       <c r="D4" s="30"/>
       <c r="E4" s="27"/>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>1960</v>
+        <v>1945</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>1961</v>
+        <v>1946</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>1962</v>
+        <v>1947</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="27"/>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>1963</v>
+        <v>1948</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>1964</v>
+        <v>1949</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>1962</v>
+        <v>1947</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="27"/>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>1965</v>
+        <v>1950</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>1966</v>
+        <v>1951</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>1967</v>
+        <v>1952</v>
       </c>
       <c r="D7" s="4"/>
       <c r="E7" s="27"/>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>1968</v>
+        <v>1953</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>1969</v>
+        <v>1954</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>1970</v>
+        <v>1955</v>
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="27"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>1971</v>
+        <v>1956</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>1972</v>
+        <v>1957</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>1973</v>
+        <v>1958</v>
       </c>
       <c r="D9" s="4"/>
       <c r="E9" s="27"/>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>1974</v>
+        <v>1959</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>1975</v>
+        <v>1960</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>1976</v>
+        <v>1961</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="27"/>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>1977</v>
+        <v>1962</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>1966</v>
+        <v>1951</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>1978</v>
+        <v>1963</v>
       </c>
       <c r="D11" s="4"/>
       <c r="E11" s="27"/>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>1979</v>
+        <v>1964</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>1980</v>
+        <v>1965</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>1981</v>
+        <v>1966</v>
       </c>
       <c r="D12" s="4"/>
       <c r="E12" s="27"/>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>1982</v>
+        <v>1967</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>1966</v>
+        <v>1951</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>1983</v>
+        <v>1968</v>
       </c>
       <c r="D13" s="4"/>
       <c r="E13" s="27"/>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>1984</v>
+        <v>1969</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>1985</v>
+        <v>1970</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>1986</v>
+        <v>1971</v>
       </c>
       <c r="D14" s="4"/>
       <c r="E14" s="27"/>
@@ -26734,61 +26694,61 @@
         <v>233</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>1987</v>
+        <v>1972</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>1988</v>
+        <v>1973</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="27"/>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>1989</v>
+        <v>1974</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>1990</v>
+        <v>1975</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>1991</v>
+        <v>1976</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>1992</v>
+        <v>1977</v>
       </c>
       <c r="E16" s="27"/>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>1993</v>
+        <v>1978</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>1994</v>
+        <v>1979</v>
       </c>
       <c r="C17" s="4"/>
       <c r="D17" s="3" t="s">
-        <v>1992</v>
+        <v>1977</v>
       </c>
       <c r="E17" s="27"/>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>1995</v>
+        <v>1980</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>1994</v>
+        <v>1979</v>
       </c>
       <c r="C18" s="4"/>
       <c r="D18" s="3" t="s">
-        <v>1992</v>
+        <v>1977</v>
       </c>
       <c r="E18" s="27"/>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>1996</v>
+        <v>1981</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>1997</v>
+        <v>1982</v>
       </c>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -26799,33 +26759,33 @@
         <v>354</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>1998</v>
+        <v>1983</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>1999</v>
+        <v>1984</v>
       </c>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>2000</v>
+        <v>1985</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>2001</v>
+        <v>1986</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>2002</v>
+        <v>1987</v>
       </c>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>2003</v>
+        <v>1988</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>2004</v>
+        <v>1989</v>
       </c>
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
@@ -26833,35 +26793,35 @@
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>2005</v>
+        <v>1990</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>2006</v>
+        <v>1991</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>2007</v>
+        <v>1992</v>
       </c>
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>2008</v>
+        <v>1993</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="3" t="s">
-        <v>2009</v>
+        <v>1994</v>
       </c>
       <c r="D24" s="4"/>
       <c r="E24" s="4"/>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>2010</v>
+        <v>1995</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="3" t="s">
-        <v>2011</v>
+        <v>1996</v>
       </c>
       <c r="D25" s="4"/>
       <c r="E25" s="4"/>
@@ -26871,10 +26831,10 @@
         <v>285</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>2012</v>
+        <v>1997</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>2013</v>
+        <v>1998</v>
       </c>
       <c r="D26" s="4"/>
       <c r="E26" s="4"/>
@@ -26884,10 +26844,10 @@
         <v>339</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>2012</v>
+        <v>1997</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>2014</v>
+        <v>1999</v>
       </c>
       <c r="D27" s="4"/>
       <c r="E27" s="4"/>
@@ -26897,49 +26857,49 @@
         <v>705</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>2015</v>
+        <v>2000</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>2016</v>
+        <v>2001</v>
       </c>
       <c r="D28" s="4"/>
       <c r="E28" s="4"/>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>2017</v>
+        <v>2002</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>2015</v>
+        <v>2000</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>2018</v>
+        <v>2003</v>
       </c>
       <c r="D29" s="4"/>
       <c r="E29" s="4"/>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>2019</v>
+        <v>2004</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>2015</v>
+        <v>2000</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>2020</v>
+        <v>2005</v>
       </c>
       <c r="D30" s="4"/>
       <c r="E30" s="4"/>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>2021</v>
+        <v>2006</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>2015</v>
+        <v>2000</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>2022</v>
+        <v>2007</v>
       </c>
       <c r="D31" s="4"/>
       <c r="E31" s="4"/>
@@ -26953,7 +26913,7 @@
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="25" t="s">
-        <v>2023</v>
+        <v>2008</v>
       </c>
       <c r="B33" s="25"/>
       <c r="C33" s="25"/>
@@ -26962,103 +26922,103 @@
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="28" t="s">
-        <v>1953</v>
+        <v>1938</v>
       </c>
       <c r="B34" s="28" t="s">
-        <v>1954</v>
+        <v>1939</v>
       </c>
       <c r="C34" s="28" t="s">
-        <v>1955</v>
+        <v>1940</v>
       </c>
       <c r="D34" s="28" t="s">
-        <v>1956</v>
+        <v>1941</v>
       </c>
       <c r="E34" s="31"/>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="29" t="s">
-        <v>2024</v>
+        <v>2009</v>
       </c>
       <c r="B35" s="29" t="s">
-        <v>2025</v>
+        <v>2010</v>
       </c>
       <c r="C35" s="29" t="s">
-        <v>2026</v>
+        <v>2011</v>
       </c>
       <c r="D35" s="29" t="s">
-        <v>2027</v>
+        <v>2012</v>
       </c>
       <c r="E35" s="4"/>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>1763</v>
+        <v>1748</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>2028</v>
+        <v>2013</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>2029</v>
+        <v>2014</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>2027</v>
+        <v>2012</v>
       </c>
       <c r="E36" s="4"/>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
-        <v>2030</v>
+        <v>2015</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>2031</v>
+        <v>2016</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>2032</v>
+        <v>2017</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>1992</v>
+        <v>1977</v>
       </c>
       <c r="E37" s="4"/>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>2033</v>
+        <v>2018</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>2034</v>
+        <v>2019</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>2034</v>
+        <v>2019</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>2035</v>
+        <v>2020</v>
       </c>
       <c r="E38" s="4"/>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>2036</v>
+        <v>2021</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>2037</v>
+        <v>2022</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>2038</v>
+        <v>2023</v>
       </c>
       <c r="D39" s="32" t="s">
-        <v>2039</v>
+        <v>2024</v>
       </c>
       <c r="E39" s="4"/>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>2040</v>
+        <v>2025</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>2041</v>
+        <v>2026</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>2042</v>
+        <v>2027</v>
       </c>
       <c r="D40" s="32"/>
       <c r="E40" s="4"/>

</xml_diff>